<commit_message>
Add PDF page-count validation and redesigned interface
</commit_message>
<xml_diff>
--- a/test_output/validation_report_with_word.xlsx
+++ b/test_output/validation_report_with_word.xlsx
@@ -14,23 +14,27 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excel rows not matched" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Word vs Excel Summary" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Word vs Excel Details" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracted Word values" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Word candidate rows" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excel rows not in Word" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run info" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Word page count" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracted Word values" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Word template info" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Word candidate rows" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excel rows not in Word" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run info" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed comparison'!$A$1:$J$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Extracted PDF values'!$A$1:$H$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Extracted PDF values'!$A$1:$I$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Candidate rows'!$A$1:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Excel rows not matched'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Word vs Excel Summary'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Word vs Excel Summary'!$A$1:$P$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Word vs Excel Details'!$A$1:$J$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Extracted Word values'!$A$1:$E$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Word candidate rows'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Excel rows not in Word'!$A$1:$H$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Run info'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Word page count'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Extracted Word values'!$A$1:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Word template info'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Word candidate rows'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Excel rows not in Word'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Run info'!$A$1:$B$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,20 +516,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -541,45 +546,50 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Total PDF pages</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Excel row</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PDF DOK-ID</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Expected Ausgabe</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PDF Ausgabe raw</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>PDF Ausgabe normalized</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Detected table</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Row start</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Issues</t>
         </is>
@@ -597,38 +607,41 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="E2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>DOC-001</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>07-2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>07.2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="J2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>All checks passed after normalization.</t>
         </is>
@@ -646,38 +659,41 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="E3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>DOC-001</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>07-2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>08.2026</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="J3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Ausgabe differs from expected input.</t>
         </is>
@@ -695,38 +711,41 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="E4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>DOC-002</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>07-2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>07/2026</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="J4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Mismatching Excel fields: Artikelnummer</t>
         </is>
@@ -744,38 +763,41 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="E5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>DOC-DOES-NOT-EXIST</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>07-2026</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="J5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>DOK-ID from PDF is empty or not present in Excel, but another row strongly matches other fields.; Fallback row found, but some Excel fields still differ: DOK-ID</t>
         </is>
@@ -793,50 +815,225 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="E6" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>DOC-DUP</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>07-2026</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Juli 2026</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="J6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>DOK-ID appears 2 times; best duplicate row selected.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K6"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Extraction mode</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>custom_mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Template type</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Custom Word mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Table index zero-based</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Header rows zero-based</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Data start row zero-based</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Mapped columns zero-based</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>{"sprache": 0, "dokumentnummer": 1, "dok_id": 2, "freigabe": 3, "artikelnummer": 4, "revision": 5, "version": 6}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Top-right Number raw</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Top-right Number normalized</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Warnings</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Word file</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Word row</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate Excel row</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate score</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -983,13 +1180,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1047,17 +1244,19 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PDF files processed</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>5</v>
+          <t>PDF folder provided</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Excel records loaded</t>
+          <t>PDF files processed</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -1067,71 +1266,113 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Word comparison</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Enabled</t>
-        </is>
+          <t>Excel records loaded</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Word file</t>
+          <t>Word comparison</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>word_list.docx</t>
+          <t>Enabled</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Word rows processed</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>3</v>
+          <t>Word file</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>word_list.docx</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Word table index zero-based</t>
+          <t>Word rows processed</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Word data start row zero-based</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>1</v>
+          <t>Word extraction mode</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>custom_mapping</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Word template type</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Custom Word mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Word table index zero-based</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Word data start row zero-based</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Word mapped columns zero-based</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>{"sprache": 0, "dokumentnummer": 1, "dok_id": 2, "freigabe": 3, "artikelnummer": 4, "revision": 5, "version": 6}</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Word top-right Number</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3211,17 +3452,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3232,35 +3474,40 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Total PDF pages</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Metadata page</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Row start</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Raw value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Normalized value</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Warnings/Error</t>
         </is>
@@ -3276,27 +3523,30 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Sprache</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>de DE _</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3308,27 +3558,30 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Dokumentnummer</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>DN-100</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>dn-100</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3340,27 +3593,30 @@
         <v>2</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>DOK-ID</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>DOC-001</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>doc-001</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3372,27 +3628,30 @@
         <v>2</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>FR-1</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>fr-1</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3404,27 +3663,30 @@
         <v>2</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Artikelnummer</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>ART-123</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>art-123</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3436,27 +3698,30 @@
         <v>2</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3468,27 +3733,30 @@
         <v>2</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3500,27 +3768,30 @@
         <v>2</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>07.2026</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3532,27 +3803,30 @@
         <v>2</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Sprache</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>en US _</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3564,27 +3838,30 @@
         <v>2</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Dokumentnummer</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>DN-200</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>dn-200</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3596,27 +3873,30 @@
         <v>2</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>DOK-ID</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>DOC-002</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>doc-002</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3628,27 +3908,30 @@
         <v>2</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>FR-2</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>fr-2</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3660,27 +3943,30 @@
         <v>2</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Artikelnummer</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>WRONG-ARTICLE</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>wrong-article</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3692,27 +3978,30 @@
         <v>2</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3724,27 +4013,30 @@
         <v>2</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3756,27 +4048,30 @@
         <v>2</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>07/2026</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3788,27 +4083,30 @@
         <v>2</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Sprache</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>fr FR _</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>fr</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3820,27 +4118,30 @@
         <v>2</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Dokumentnummer</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>DN-400</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>dn-400</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3852,27 +4153,30 @@
         <v>2</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>DOK-ID</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>DOC-DOES-NOT-EXIST</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>doc-does-not-exist</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3884,27 +4188,30 @@
         <v>2</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>FR-5</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>fr-5</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3916,27 +4223,30 @@
         <v>2</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Artikelnummer</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>ART-555</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>art-555</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3948,27 +4258,30 @@
         <v>2</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3980,27 +4293,30 @@
         <v>2</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4012,27 +4328,30 @@
         <v>2</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4044,27 +4363,30 @@
         <v>2</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Sprache</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>de DE _</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4076,27 +4398,30 @@
         <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Dokumentnummer</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>DN-300</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>dn-300</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4108,27 +4433,30 @@
         <v>2</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>DOK-ID</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>DOC-DUP</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>doc-dup</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4140,27 +4468,30 @@
         <v>2</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>FR-3</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>fr-3</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4172,27 +4503,30 @@
         <v>2</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Artikelnummer</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>ART-333</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>art-333</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4204,27 +4538,30 @@
         <v>2</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4236,27 +4573,30 @@
         <v>2</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4268,27 +4608,30 @@
         <v>2</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Juli 2026</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4300,27 +4643,30 @@
         <v>2</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Sprache</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>de DE _</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4332,27 +4678,30 @@
         <v>2</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Dokumentnummer</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>DN-100</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>dn-100</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4364,27 +4713,30 @@
         <v>2</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>DOK-ID</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>DOC-001</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>doc-001</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4396,27 +4748,30 @@
         <v>2</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>FR-1</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>fr-1</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4428,27 +4783,30 @@
         <v>2</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Artikelnummer</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>ART-123</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>art-123</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4460,27 +4818,30 @@
         <v>2</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4492,27 +4853,30 @@
         <v>2</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4524,30 +4888,33 @@
         <v>2</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>08.2026</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H41"/>
+  <autoFilter ref="A1:I41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4834,18 +5201,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4861,24 +5235,24 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Overall status</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Word/Excel status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Excel row</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Word DOK-ID</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Word Dok.-Nr.</t>
@@ -4890,6 +5264,41 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Word Rev. neu</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Word Vers. neu</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Word Number</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Word Blatt/sheets</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Matched PDF</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Actual PDF pages</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Page-count result</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Issues</t>
         </is>
@@ -4909,17 +5318,17 @@
           <t>WORD_OK</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>WORD_OK</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>DOC-001</t>
-        </is>
-      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>DN-100</t>
@@ -4930,7 +5339,34 @@
           <t>ART-123</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>FR-1</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>WORD_PAGE_COUNT_MISSING</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>The Word Blatt / sheets cell is empty.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4946,17 +5382,17 @@
           <t>WORD_OK</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>WORD_OK</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>DOC-002</t>
-        </is>
-      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>DN-200</t>
@@ -4967,7 +5403,34 @@
           <t>ART-222</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>FR-2</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>WORD_PAGE_COUNT_MISSING</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>The Word Blatt / sheets cell is empty.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4983,17 +5446,17 @@
           <t>WORD_LIKELY_WRONG_DOK_ID</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>WORD_LIKELY_WRONG_DOK_ID</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>DOC-WRONG</t>
-        </is>
-      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>DN-400</t>
@@ -5006,12 +5469,35 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID from Word is empty or not present in Excel, but another row strongly matches other fields.; Matched row still has mismatching fields: DOK-ID</t>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>FR-5</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>WORD_PAGE_COUNT_MISSING</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>The Word DOK-ID is not present in Excel, but Dokument-Nr. uniquely identifies the row.; The Word Blatt / sheets cell is empty.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
+  <autoFilter ref="A1:P4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5108,27 +5594,27 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sprache</t>
+          <t>Dokumentnummer</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>DN-100</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>dn-100</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>DN-100</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>dn-100</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -5156,27 +5642,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Dokumentnummer</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>DN-100</t>
+          <t>ART-123</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>dn-100</t>
+          <t>art-123</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>DN-100</t>
+          <t>ART-123</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>dn-100</t>
+          <t>art-123</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -5204,27 +5690,27 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID</t>
+          <t>Revision</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>doc-001</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>doc-001</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -5252,27 +5738,27 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Freigabe-/Änd.-Nr.</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>FR-1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>fr-1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>FR-1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>fr-1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -5300,27 +5786,27 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>ART-123</t>
+          <t>FR-1</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>art-123</t>
+          <t>fr-1</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>ART-123</t>
+          <t>FR-1</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>art-123</t>
+          <t>fr-1</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -5348,27 +5834,27 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Revision</t>
+          <t>DOK-ID</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>DOC-001</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>doc-001</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>DOC-001</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>doc-001</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -5396,27 +5882,27 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Sprache</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>de</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>de</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>de</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -5444,27 +5930,27 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sprache</t>
+          <t>Dokumentnummer</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>DN-200</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>dn-200</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>DN-200</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>dn-200</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -5492,27 +5978,27 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dokumentnummer</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>DN-200</t>
+          <t>ART-222</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>dn-200</t>
+          <t>art-222</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>DN-200</t>
+          <t>ART-222</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>dn-200</t>
+          <t>art-222</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -5540,27 +6026,27 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID</t>
+          <t>Revision</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>DOC-002</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>doc-002</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>DOC-002</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>doc-002</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -5588,27 +6074,27 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Freigabe-/Änd.-Nr.</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>FR-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>fr-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>FR-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>fr-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -5636,27 +6122,27 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>ART-222</t>
+          <t>FR-2</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>art-222</t>
+          <t>fr-2</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>ART-222</t>
+          <t>FR-2</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>art-222</t>
+          <t>fr-2</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -5684,27 +6170,27 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Revision</t>
+          <t>DOK-ID</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>DOC-002</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>doc-002</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>DOC-002</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>doc-002</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -5732,27 +6218,27 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Sprache</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>en</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>en</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>en</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>en</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -5780,27 +6266,27 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Sprache</t>
+          <t>Dokumentnummer</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>DN-400</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>dn-400</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>DN-400</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>dn-400</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -5828,27 +6314,27 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Dokumentnummer</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>DN-400</t>
+          <t>ART-555</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>dn-400</t>
+          <t>art-555</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>DN-400</t>
+          <t>ART-555</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>dn-400</t>
+          <t>art-555</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -5876,32 +6362,32 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID</t>
+          <t>Revision</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>DOC-WRONG</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>doc-wrong</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>DOC-004</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>doc-004</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -5924,27 +6410,27 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Freigabe-/Änd.-Nr.</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>FR-5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>fr-5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>FR-5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>fr-5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -5972,27 +6458,27 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>ART-555</t>
+          <t>FR-5</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>art-555</t>
+          <t>fr-5</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ART-555</t>
+          <t>FR-5</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>art-555</t>
+          <t>fr-5</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -6020,32 +6506,32 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Revision</t>
+          <t>DOK-ID</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>DOC-WRONG</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>doc-wrong</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>DOC-004</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>doc-004</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -6068,27 +6554,27 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Sprache</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -6104,6 +6590,181 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Word file</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Word row</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Excel row</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Dok.-Nr.</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Word Blatt/sheets raw</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Word pages normalized</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Matched PDF</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Actual PDF pages</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>word_list.docx</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>DN-100</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>WORD_PAGE_COUNT_MISSING</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>The Word Blatt / sheets cell is empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>word_list.docx</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>DN-200</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>WORD_PAGE_COUNT_MISSING</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>The Word Blatt / sheets cell is empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>word_list.docx</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>DN-400</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>WORD_PAGE_COUNT_MISSING</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>The Word Blatt / sheets cell is empty.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6157,17 +6818,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Sprache</t>
+          <t>Dokumentnummer</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>DN-100</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>dn-100</t>
         </is>
       </c>
     </row>
@@ -6182,17 +6843,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Dokumentnummer</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>DN-100</t>
+          <t>ART-123</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>dn-100</t>
+          <t>art-123</t>
         </is>
       </c>
     </row>
@@ -6207,17 +6868,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID</t>
+          <t>Revision</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>doc-001</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6232,17 +6893,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Freigabe-/Änd.-Nr.</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>FR-1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>fr-1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6257,17 +6918,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ART-123</t>
+          <t>FR-1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>art-123</t>
+          <t>fr-1</t>
         </is>
       </c>
     </row>
@@ -6282,17 +6943,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Revision</t>
+          <t>DOK-ID</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>DOC-001</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>doc-001</t>
         </is>
       </c>
     </row>
@@ -6307,17 +6968,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Sprache</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>de</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>de</t>
         </is>
       </c>
     </row>
@@ -6332,17 +6993,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sprache</t>
+          <t>Dokumentnummer</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>DN-200</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>dn-200</t>
         </is>
       </c>
     </row>
@@ -6357,17 +7018,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Dokumentnummer</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>DN-200</t>
+          <t>ART-222</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>dn-200</t>
+          <t>art-222</t>
         </is>
       </c>
     </row>
@@ -6382,17 +7043,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID</t>
+          <t>Revision</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>DOC-002</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>doc-002</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6407,17 +7068,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Freigabe-/Änd.-Nr.</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>FR-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>fr-2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6432,17 +7093,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ART-222</t>
+          <t>FR-2</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>art-222</t>
+          <t>fr-2</t>
         </is>
       </c>
     </row>
@@ -6457,17 +7118,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Revision</t>
+          <t>DOK-ID</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>DOC-002</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>doc-002</t>
         </is>
       </c>
     </row>
@@ -6482,17 +7143,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Sprache</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>en</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>en</t>
         </is>
       </c>
     </row>
@@ -6507,17 +7168,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Sprache</t>
+          <t>Dokumentnummer</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>DN-400</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>dn-400</t>
         </is>
       </c>
     </row>
@@ -6532,17 +7193,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Dokumentnummer</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>DN-400</t>
+          <t>ART-555</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>dn-400</t>
+          <t>art-555</t>
         </is>
       </c>
     </row>
@@ -6557,17 +7218,17 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>DOK-ID</t>
+          <t>Revision</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>DOC-WRONG</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>doc-wrong</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -6582,17 +7243,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Freigabe-/Änd.-Nr.</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>FR-5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>fr-5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6607,17 +7268,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Freigabe-/Änd.-Nr.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ART-555</t>
+          <t>FR-5</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>art-555</t>
+          <t>fr-5</t>
         </is>
       </c>
     </row>
@@ -6632,17 +7293,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Revision</t>
+          <t>DOK-ID</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>DOC-WRONG</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>doc-wrong</t>
         </is>
       </c>
     </row>
@@ -6657,17 +7318,17 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Sprache</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>fr</t>
         </is>
       </c>
     </row>
@@ -6675,158 +7336,4 @@
   <autoFilter ref="A1:E22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Word file</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Word row</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Candidate Excel row</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Candidate score</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>word_list.docx</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>WORD_LIKELY_WRONG_DOK_ID</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>word_list.docx</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>WORD_LIKELY_WRONG_DOK_ID</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>8.300000000000001</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>word_list.docx</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>WORD_LIKELY_WRONG_DOK_ID</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>word_list.docx</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>WORD_LIKELY_WRONG_DOK_ID</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>word_list.docx</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>WORD_LIKELY_WRONG_DOK_ID</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E6"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>